<commit_message>
Adding 2022 trade data
</commit_message>
<xml_diff>
--- a/data/trade_balances.xlsx
+++ b/data/trade_balances.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\My PC (LAPTOP-IKUHQKMA)\Documents\GitHub\russia_sentiment_paper\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skybl\Dropbox\My PC (LAPTOP-IKUHQKMA)\Documents\GitHub\russia_sentiment_paper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C535AB5-21AB-4510-9CB8-1A4630A700BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87589DB4-B846-48F5-B027-8027DA12E289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FCB7CB41-B692-436C-843A-4F17D898C438}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FCB7CB41-B692-436C-843A-4F17D898C438}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="2021" sheetId="1" r:id="rId1"/>
+    <sheet name="2022" sheetId="2" r:id="rId2"/>
+    <sheet name="2023" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="17">
   <si>
     <t>Belarus</t>
   </si>
@@ -79,12 +81,21 @@
   <si>
     <t>https://wits.worldbank.org/CountryProfile/en/Country/ARM/Year/2021/TradeFlow/EXPIMP/Partner/all</t>
   </si>
+  <si>
+    <t>CSTO in Sample</t>
+  </si>
+  <si>
+    <t>West Percent</t>
+  </si>
+  <si>
+    <t>Russia Percent</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,6 +106,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -117,15 +136,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -459,10 +481,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55A2B9CC-AEAF-44AF-A535-5339582CC0B7}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -484,8 +506,35 @@
       <c r="G1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -509,8 +558,38 @@
         <f>F2/E2</f>
         <v>0.21845621599939832</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="1">
+        <f>C2/E2</f>
+        <v>0.35027200481335707</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>23130</v>
+      </c>
+      <c r="L2">
+        <v>18494</v>
+      </c>
+      <c r="M2">
+        <v>2324</v>
+      </c>
+      <c r="N2">
+        <v>1897</v>
+      </c>
+      <c r="O2">
+        <v>492314</v>
+      </c>
+      <c r="P2">
+        <f>K2+L2+M2+N2</f>
+        <v>45845</v>
+      </c>
+      <c r="Q2">
+        <f>P2/O2</f>
+        <v>9.3121463131253635E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -534,21 +613,51 @@
         <f t="shared" ref="G3:G4" si="1">F3/E3</f>
         <v>0.22931764368228458</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H4" si="2">C3/E3</f>
+        <v>0.28578603716725265</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>15636</v>
+      </c>
+      <c r="L3">
+        <v>7132</v>
+      </c>
+      <c r="M3">
+        <v>1032</v>
+      </c>
+      <c r="N3">
+        <v>712</v>
+      </c>
+      <c r="O3">
+        <v>293497</v>
+      </c>
+      <c r="P3">
+        <f>K3+L3+M3+N3</f>
+        <v>24512</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q4" si="3">P3/O3</f>
+        <v>8.351703765285505E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
-        <f t="shared" ref="B4:D4" si="2">SUM(B2:B3)</f>
+        <f t="shared" ref="B4:D4" si="4">SUM(B2:B3)</f>
         <v>43605</v>
       </c>
       <c r="C4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>25921</v>
       </c>
       <c r="D4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>618</v>
       </c>
       <c r="E4">
@@ -563,8 +672,43 @@
         <f t="shared" si="1"/>
         <v>0.22401468788249693</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="1">
+        <f t="shared" si="2"/>
+        <v>0.31727050183598532</v>
+      </c>
+      <c r="J4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:N4" si="5">SUM(K2:K3)</f>
+        <v>38766</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="5"/>
+        <v>25626</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="5"/>
+        <v>3356</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="5"/>
+        <v>2609</v>
+      </c>
+      <c r="O4">
+        <f>SUM(O2:O3)</f>
+        <v>785811</v>
+      </c>
+      <c r="P4">
+        <f>K4+L4+M4+N4</f>
+        <v>70357</v>
+      </c>
+      <c r="Q4" s="1">
+        <f t="shared" si="3"/>
+        <v>8.9534251874814688E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -586,8 +730,11 @@
       <c r="G6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -611,8 +758,12 @@
         <f>F7/E7</f>
         <v>0.58883717424485105</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="1">
+        <f>C7/E7</f>
+        <v>0.1322617724095046</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -629,28 +780,32 @@
         <v>27752</v>
       </c>
       <c r="F8">
-        <f t="shared" ref="F8:F9" si="3">B8-C8+D8</f>
+        <f t="shared" ref="F8:F9" si="6">B8-C8+D8</f>
         <v>6328</v>
       </c>
       <c r="G8">
-        <f t="shared" ref="G8:G9" si="4">F8/E8</f>
+        <f t="shared" ref="G8:G9" si="7">F8/E8</f>
         <v>0.22801960219083309</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="1">
+        <f t="shared" ref="H8:H9" si="8">C8/E8</f>
+        <v>0.63436869414816954</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
       <c r="B9">
-        <f t="shared" ref="B9" si="5">SUM(B7:B8)</f>
+        <f t="shared" ref="B9" si="9">SUM(B7:B8)</f>
         <v>60601</v>
       </c>
       <c r="C9">
-        <f t="shared" ref="C9" si="6">SUM(C7:C8)</f>
+        <f t="shared" ref="C9" si="10">SUM(C7:C8)</f>
         <v>24624</v>
       </c>
       <c r="D9">
-        <f t="shared" ref="D9" si="7">SUM(D7:D8)</f>
+        <f t="shared" ref="D9" si="11">SUM(D7:D8)</f>
         <v>1600</v>
       </c>
       <c r="E9">
@@ -658,15 +813,19 @@
         <v>80821</v>
       </c>
       <c r="F9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>37577</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.46494104255082219</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="1">
+        <f t="shared" si="8"/>
+        <v>0.30467329035770407</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -688,8 +847,11 @@
       <c r="G11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -713,8 +875,1507 @@
         <f>F12/E12</f>
         <v>0.82987346332237588</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="1">
+        <f>C12/E12</f>
+        <v>4.1473409285360474E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>7562</v>
+      </c>
+      <c r="C13">
+        <v>2073</v>
+      </c>
+      <c r="D13">
+        <v>454</v>
+      </c>
+      <c r="E13">
+        <v>11696</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:F14" si="12">B13-C13+D13</f>
+        <v>5943</v>
+      </c>
+      <c r="G13">
+        <f t="shared" ref="G13:G14" si="13">F13/E13</f>
+        <v>0.50812243502051979</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" ref="H13:H14" si="14">C13/E13</f>
+        <v>0.17724008207934336</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <f t="shared" ref="B14" si="15">SUM(B12:B13)</f>
+        <v>26615</v>
+      </c>
+      <c r="C14">
+        <f t="shared" ref="C14" si="16">SUM(C12:C13)</f>
+        <v>2994</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ref="D14" si="17">SUM(D12:D13)</f>
+        <v>751</v>
+      </c>
+      <c r="E14">
+        <f>SUM(E12:E13)</f>
+        <v>33903</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="12"/>
+        <v>24372</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="13"/>
+        <v>0.71887443589062916</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" si="14"/>
+        <v>8.831076895849925E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" t="s">
+        <v>9</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17">
+        <v>1973</v>
+      </c>
+      <c r="C17">
+        <v>794</v>
+      </c>
+      <c r="D17">
+        <v>86</v>
+      </c>
+      <c r="E17">
+        <v>2965</v>
+      </c>
+      <c r="F17">
+        <f>B17-C17+D17</f>
+        <v>1265</v>
+      </c>
+      <c r="G17">
+        <f>F17/E17</f>
+        <v>0.42664418212478922</v>
+      </c>
+      <c r="H17" s="1">
+        <f>C17/E17</f>
+        <v>0.26779089376053961</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>3203</v>
+      </c>
+      <c r="C18">
+        <v>1785</v>
+      </c>
+      <c r="D18">
+        <v>127</v>
+      </c>
+      <c r="E18">
+        <v>5324</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18:F19" si="18">B18-C18+D18</f>
+        <v>1545</v>
+      </c>
+      <c r="G18">
+        <f t="shared" ref="G18:G19" si="19">F18/E18</f>
+        <v>0.29019534184823442</v>
+      </c>
+      <c r="H18" s="1">
+        <f t="shared" ref="H18:H19" si="20">C18/E18</f>
+        <v>0.33527422990232908</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19">
+        <f t="shared" ref="B19" si="21">SUM(B17:B18)</f>
+        <v>5176</v>
+      </c>
+      <c r="C19">
+        <f t="shared" ref="C19" si="22">SUM(C17:C18)</f>
+        <v>2579</v>
+      </c>
+      <c r="D19">
+        <f t="shared" ref="D19" si="23">SUM(D17:D18)</f>
+        <v>213</v>
+      </c>
+      <c r="E19">
+        <f>SUM(E17:E18)</f>
+        <v>8289</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="18"/>
+        <v>2810</v>
+      </c>
+      <c r="G19" s="1">
+        <f t="shared" si="19"/>
+        <v>0.33900349861261914</v>
+      </c>
+      <c r="H19" s="1">
+        <f t="shared" si="20"/>
+        <v>0.31113523947400168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G20" s="1"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A22" r:id="rId1" xr:uid="{054DAB19-AF0C-4AD8-A1D1-E4794718B406}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A09AFB8C-C702-4CB1-8C3A-A823CE50EEC1}">
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>22500</v>
+      </c>
+      <c r="C2">
+        <v>13972</v>
+      </c>
+      <c r="D2">
+        <v>186</v>
+      </c>
+      <c r="E2">
+        <v>39889</v>
+      </c>
+      <c r="F2">
+        <f>B2-C2+D2</f>
+        <v>8714</v>
+      </c>
+      <c r="G2" s="1">
+        <f>F2/E2</f>
+        <v>0.21845621599939832</v>
+      </c>
+      <c r="H2" s="1">
+        <f>C2/E2</f>
+        <v>0.35027200481335707</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>23130</v>
+      </c>
+      <c r="L2">
+        <v>18494</v>
+      </c>
+      <c r="M2">
+        <v>2324</v>
+      </c>
+      <c r="N2">
+        <v>1897</v>
+      </c>
+      <c r="O2">
+        <v>492314</v>
+      </c>
+      <c r="P2">
+        <f>K2+L2+M2+N2</f>
+        <v>45845</v>
+      </c>
+      <c r="Q2">
+        <f>P2/O2</f>
+        <v>9.3121463131253635E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>21105</v>
+      </c>
+      <c r="C3">
+        <v>11949</v>
+      </c>
+      <c r="D3">
+        <v>432</v>
+      </c>
+      <c r="E3">
+        <v>41811</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F4" si="0">B3-C3+D3</f>
+        <v>9588</v>
+      </c>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G4" si="1">F3/E3</f>
+        <v>0.22931764368228458</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H4" si="2">C3/E3</f>
+        <v>0.28578603716725265</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>15636</v>
+      </c>
+      <c r="L3">
+        <v>7132</v>
+      </c>
+      <c r="M3">
+        <v>1032</v>
+      </c>
+      <c r="N3">
+        <v>712</v>
+      </c>
+      <c r="O3">
+        <v>293497</v>
+      </c>
+      <c r="P3">
+        <f>K3+L3+M3+N3</f>
+        <v>24512</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q4" si="3">P3/O3</f>
+        <v>8.351703765285505E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <f t="shared" ref="B4:D4" si="4">SUM(B2:B3)</f>
+        <v>43605</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="4"/>
+        <v>25921</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="4"/>
+        <v>618</v>
+      </c>
+      <c r="E4">
+        <f>SUM(E2:E3)</f>
+        <v>81700</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>18302</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="1"/>
+        <v>0.22401468788249693</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" si="2"/>
+        <v>0.31727050183598532</v>
+      </c>
+      <c r="J4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:N4" si="5">SUM(K2:K3)</f>
+        <v>38766</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="5"/>
+        <v>25626</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="5"/>
+        <v>3356</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="5"/>
+        <v>2609</v>
+      </c>
+      <c r="O4">
+        <f>SUM(O2:O3)</f>
+        <v>785811</v>
+      </c>
+      <c r="P4">
+        <f>K4+L4+M4+N4</f>
+        <v>70357</v>
+      </c>
+      <c r="Q4" s="1">
+        <f t="shared" si="3"/>
+        <v>8.9534251874814688E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" t="s">
+        <v>4</v>
+      </c>
+      <c r="L6" t="s">
+        <v>5</v>
+      </c>
+      <c r="M6" t="s">
+        <v>6</v>
+      </c>
+      <c r="N6" t="s">
+        <v>7</v>
+      </c>
+      <c r="O6" t="s">
+        <v>8</v>
+      </c>
+      <c r="P6" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>50591</v>
+      </c>
+      <c r="C7">
+        <v>8781</v>
+      </c>
+      <c r="D7">
+        <v>1704</v>
+      </c>
+      <c r="E7">
+        <v>76140</v>
+      </c>
+      <c r="F7">
+        <f>B7-C7+D7</f>
+        <v>43514</v>
+      </c>
+      <c r="G7" s="1">
+        <f>F7/E7</f>
+        <v>0.57149986866298919</v>
+      </c>
+      <c r="H7" s="1">
+        <f>C7/E7</f>
+        <v>0.11532702915681639</v>
+      </c>
+      <c r="J7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <f>B7-'2021'!B7</f>
+        <v>13485</v>
+      </c>
+      <c r="L7">
+        <f>C7-'2021'!C7</f>
+        <v>1762</v>
+      </c>
+      <c r="M7">
+        <f>D7-'2021'!D7</f>
+        <v>542</v>
+      </c>
+      <c r="N7">
+        <f>E7-'2021'!E7</f>
+        <v>23071</v>
+      </c>
+      <c r="O7">
+        <f>K7-L7+M7</f>
+        <v>12265</v>
+      </c>
+      <c r="P7" s="1">
+        <f>G7-'2021'!G7</f>
+        <v>-1.7337305581861862E-2</v>
+      </c>
+      <c r="Q7" s="1">
+        <f>H7-'2021'!H7</f>
+        <v>-1.6934743252688206E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>24851</v>
+      </c>
+      <c r="C8">
+        <v>17343</v>
+      </c>
+      <c r="D8">
+        <v>555</v>
+      </c>
+      <c r="E8">
+        <v>30952</v>
+      </c>
+      <c r="F8">
+        <f t="shared" ref="F8:F9" si="6">B8-C8+D8</f>
+        <v>8063</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" ref="G8:G9" si="7">F8/E8</f>
+        <v>0.26050012923235977</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" ref="H8:H9" si="8">C8/E8</f>
+        <v>0.56031920392866374</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <f>B8-'2021'!B8</f>
+        <v>1356</v>
+      </c>
+      <c r="L8">
+        <f>C8-'2021'!C8</f>
+        <v>-262</v>
+      </c>
+      <c r="M8">
+        <f>D8-'2021'!D8</f>
+        <v>117</v>
+      </c>
+      <c r="N8">
+        <f>E8-'2021'!E8</f>
+        <v>3200</v>
+      </c>
+      <c r="O8">
+        <f t="shared" ref="O8:O9" si="9">K8-L8+M8</f>
+        <v>1735</v>
+      </c>
+      <c r="P8" s="1">
+        <f>G8-'2021'!G8</f>
+        <v>3.248052704152668E-2</v>
+      </c>
+      <c r="Q8" s="1">
+        <f>H8-'2021'!H8</f>
+        <v>-7.4049490219505798E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <f t="shared" ref="B9:D9" si="10">SUM(B7:B8)</f>
+        <v>75442</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="10"/>
+        <v>26124</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="10"/>
+        <v>2259</v>
+      </c>
+      <c r="E9">
+        <f>SUM(E7:E8)</f>
+        <v>107092</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="6"/>
+        <v>51577</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="7"/>
+        <v>0.48161393941657638</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="8"/>
+        <v>0.24393979008702799</v>
+      </c>
+      <c r="J9" t="s">
+        <v>3</v>
+      </c>
+      <c r="K9">
+        <f t="shared" ref="K9:M9" si="11">SUM(K7:K8)</f>
+        <v>14841</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="11"/>
+        <v>1500</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="11"/>
+        <v>659</v>
+      </c>
+      <c r="N9">
+        <f>SUM(N7:N8)</f>
+        <v>26271</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="9"/>
+        <v>14000</v>
+      </c>
+      <c r="P9" s="1">
+        <f>G9-'2021'!G9</f>
+        <v>1.6672896865754183E-2</v>
+      </c>
+      <c r="Q9" s="1">
+        <f>H9-'2021'!H9</f>
+        <v>-6.0733500270676088E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K11" t="s">
+        <v>4</v>
+      </c>
+      <c r="L11" t="s">
+        <v>5</v>
+      </c>
+      <c r="M11" t="s">
+        <v>6</v>
+      </c>
+      <c r="N11" t="s">
+        <v>7</v>
+      </c>
+      <c r="O11" t="s">
+        <v>8</v>
+      </c>
+      <c r="P11" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12">
+        <v>32085</v>
+      </c>
+      <c r="C12">
+        <v>975</v>
+      </c>
+      <c r="D12">
+        <v>91</v>
+      </c>
+      <c r="E12">
+        <v>38146</v>
+      </c>
+      <c r="F12">
+        <f>B12-C12+D12</f>
+        <v>31201</v>
+      </c>
+      <c r="G12" s="1">
+        <f>F12/E12</f>
+        <v>0.81793634981387298</v>
+      </c>
+      <c r="H12" s="1">
+        <f>C12/E12</f>
+        <v>2.5559691710795366E-2</v>
+      </c>
+      <c r="J12" t="s">
+        <v>2</v>
+      </c>
+      <c r="K12">
+        <f>B12-'2021'!B12</f>
+        <v>13032</v>
+      </c>
+      <c r="L12">
+        <f>C12-'2021'!C12</f>
+        <v>54</v>
+      </c>
+      <c r="M12">
+        <f>D12-'2021'!D12</f>
+        <v>-206</v>
+      </c>
+      <c r="N12">
+        <f>E12-'2021'!E12</f>
+        <v>15939</v>
+      </c>
+      <c r="O12">
+        <f>K12-L12+M12</f>
+        <v>12772</v>
+      </c>
+      <c r="P12" s="1">
+        <f>G12-'2021'!G12</f>
+        <v>-1.1937113508502906E-2</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>H12-'2021'!H12</f>
+        <v>-1.5913717574565108E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>9583</v>
+      </c>
+      <c r="C13">
+        <v>2733</v>
+      </c>
+      <c r="D13">
+        <v>492</v>
+      </c>
+      <c r="E13">
+        <v>14536</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:F14" si="12">B13-C13+D13</f>
+        <v>7342</v>
+      </c>
+      <c r="G13" s="1">
+        <f t="shared" ref="G13:G14" si="13">F13/E13</f>
+        <v>0.50509080902586678</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" ref="H13:H14" si="14">C13/E13</f>
+        <v>0.18801596037424326</v>
+      </c>
+      <c r="J13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <f>B13-'2021'!B13</f>
+        <v>2021</v>
+      </c>
+      <c r="L13">
+        <f>C13-'2021'!C13</f>
+        <v>660</v>
+      </c>
+      <c r="M13">
+        <f>D13-'2021'!D13</f>
+        <v>38</v>
+      </c>
+      <c r="N13">
+        <f>E13-'2021'!E13</f>
+        <v>2840</v>
+      </c>
+      <c r="O13">
+        <f t="shared" ref="O13:O14" si="15">K13-L13+M13</f>
+        <v>1399</v>
+      </c>
+      <c r="P13" s="1">
+        <f>G13-'2021'!G13</f>
+        <v>-3.0316259946530089E-3</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>H13-'2021'!H13</f>
+        <v>1.0775878294899899E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <f t="shared" ref="B14:D14" si="16">SUM(B12:B13)</f>
+        <v>41668</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="16"/>
+        <v>3708</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="16"/>
+        <v>583</v>
+      </c>
+      <c r="E14">
+        <f>SUM(E12:E13)</f>
+        <v>52682</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="12"/>
+        <v>38543</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="13"/>
+        <v>0.73161611176492924</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" si="14"/>
+        <v>7.038457158042595E-2</v>
+      </c>
+      <c r="J14" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14">
+        <f t="shared" ref="K14:M14" si="17">SUM(K12:K13)</f>
+        <v>15053</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="17"/>
+        <v>714</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="17"/>
+        <v>-168</v>
+      </c>
+      <c r="N14">
+        <f>SUM(N12:N13)</f>
+        <v>18779</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="15"/>
+        <v>14171</v>
+      </c>
+      <c r="P14" s="1">
+        <f>G14-'2021'!G14</f>
+        <v>1.2741675874300085E-2</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>H14-'2021'!H14</f>
+        <v>-1.79261973780733E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" t="s">
+        <v>4</v>
+      </c>
+      <c r="L16" t="s">
+        <v>5</v>
+      </c>
+      <c r="M16" t="s">
+        <v>6</v>
+      </c>
+      <c r="N16" t="s">
+        <v>7</v>
+      </c>
+      <c r="O16" t="s">
+        <v>8</v>
+      </c>
+      <c r="P16" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17">
+        <v>3818</v>
+      </c>
+      <c r="C17">
+        <v>2417</v>
+      </c>
+      <c r="D17">
+        <v>84</v>
+      </c>
+      <c r="E17">
+        <v>5364</v>
+      </c>
+      <c r="F17">
+        <f>B17-C17+D17</f>
+        <v>1485</v>
+      </c>
+      <c r="G17" s="1">
+        <f>F17/E17</f>
+        <v>0.27684563758389263</v>
+      </c>
+      <c r="H17" s="1">
+        <f>C17/E17</f>
+        <v>0.45059656972408652</v>
+      </c>
+      <c r="J17" t="s">
+        <v>2</v>
+      </c>
+      <c r="K17">
+        <f>B17-'2021'!B17</f>
+        <v>1845</v>
+      </c>
+      <c r="L17">
+        <f>C17-'2021'!C17</f>
+        <v>1623</v>
+      </c>
+      <c r="M17">
+        <f>D17-'2021'!D17</f>
+        <v>-2</v>
+      </c>
+      <c r="N17">
+        <f>E17-'2021'!E17</f>
+        <v>2399</v>
+      </c>
+      <c r="O17">
+        <f>K17-L17+M17</f>
+        <v>220</v>
+      </c>
+      <c r="P17" s="1">
+        <f>G17-'2021'!G17</f>
+        <v>-0.14979854454089658</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>H17-'2021'!H17</f>
+        <v>0.18280567596354691</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>4879</v>
+      </c>
+      <c r="C18">
+        <v>2637</v>
+      </c>
+      <c r="D18">
+        <v>398</v>
+      </c>
+      <c r="E18">
+        <v>8650</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18:F19" si="18">B18-C18+D18</f>
+        <v>2640</v>
+      </c>
+      <c r="G18" s="1">
+        <f t="shared" ref="G18:G19" si="19">F18/E18</f>
+        <v>0.30520231213872834</v>
+      </c>
+      <c r="H18" s="1">
+        <f t="shared" ref="H18:H19" si="20">C18/E18</f>
+        <v>0.30485549132947976</v>
+      </c>
+      <c r="J18" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <f>B18-'2021'!B18</f>
+        <v>1676</v>
+      </c>
+      <c r="L18">
+        <f>C18-'2021'!C18</f>
+        <v>852</v>
+      </c>
+      <c r="M18">
+        <f>D18-'2021'!D18</f>
+        <v>271</v>
+      </c>
+      <c r="N18">
+        <f>E18-'2021'!E18</f>
+        <v>3326</v>
+      </c>
+      <c r="O18">
+        <f t="shared" ref="O18:O19" si="21">K18-L18+M18</f>
+        <v>1095</v>
+      </c>
+      <c r="P18" s="1">
+        <f>G18-'2021'!G18</f>
+        <v>1.5006970290493915E-2</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>H18-'2021'!H18</f>
+        <v>-3.0418738572849324E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19">
+        <f t="shared" ref="B19:D19" si="22">SUM(B17:B18)</f>
+        <v>8697</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="22"/>
+        <v>5054</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="22"/>
+        <v>482</v>
+      </c>
+      <c r="E19">
+        <f>SUM(E17:E18)</f>
+        <v>14014</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="18"/>
+        <v>4125</v>
+      </c>
+      <c r="G19" s="1">
+        <f t="shared" si="19"/>
+        <v>0.29434850863422291</v>
+      </c>
+      <c r="H19" s="1">
+        <f t="shared" si="20"/>
+        <v>0.36063936063936064</v>
+      </c>
+      <c r="J19" t="s">
+        <v>3</v>
+      </c>
+      <c r="K19">
+        <f t="shared" ref="K19:M19" si="23">SUM(K17:K18)</f>
+        <v>3521</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="23"/>
+        <v>2475</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="23"/>
+        <v>269</v>
+      </c>
+      <c r="N19">
+        <f>SUM(N17:N18)</f>
+        <v>5725</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="21"/>
+        <v>1315</v>
+      </c>
+      <c r="P19" s="1">
+        <f>G19-'2021'!G19</f>
+        <v>-4.4654989978396231E-2</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>H19-'2021'!H19</f>
+        <v>4.9504121165358961E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A9185D-7A30-4AF2-A5D7-32A07A35B276}">
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>22500</v>
+      </c>
+      <c r="C2">
+        <v>13972</v>
+      </c>
+      <c r="D2">
+        <v>186</v>
+      </c>
+      <c r="E2">
+        <v>39889</v>
+      </c>
+      <c r="F2">
+        <f>B2-C2+D2</f>
+        <v>8714</v>
+      </c>
+      <c r="G2">
+        <f>F2/E2</f>
+        <v>0.21845621599939832</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>23130</v>
+      </c>
+      <c r="L2">
+        <v>18494</v>
+      </c>
+      <c r="M2">
+        <v>2324</v>
+      </c>
+      <c r="N2">
+        <v>1897</v>
+      </c>
+      <c r="O2">
+        <v>492314</v>
+      </c>
+      <c r="P2">
+        <f>K2+L2+M2+N2</f>
+        <v>45845</v>
+      </c>
+      <c r="Q2">
+        <f>P2/O2</f>
+        <v>9.3121463131253635E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>21105</v>
+      </c>
+      <c r="C3">
+        <v>11949</v>
+      </c>
+      <c r="D3">
+        <v>432</v>
+      </c>
+      <c r="E3">
+        <v>41811</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F4" si="0">B3-C3+D3</f>
+        <v>9588</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G4" si="1">F3/E3</f>
+        <v>0.22931764368228458</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>15636</v>
+      </c>
+      <c r="L3">
+        <v>7132</v>
+      </c>
+      <c r="M3">
+        <v>1032</v>
+      </c>
+      <c r="N3">
+        <v>712</v>
+      </c>
+      <c r="O3">
+        <v>293497</v>
+      </c>
+      <c r="P3">
+        <f>K3+L3+M3+N3</f>
+        <v>24512</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q4" si="2">P3/O3</f>
+        <v>8.351703765285505E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <f t="shared" ref="B4:D4" si="3">SUM(B2:B3)</f>
+        <v>43605</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="3"/>
+        <v>25921</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="3"/>
+        <v>618</v>
+      </c>
+      <c r="E4">
+        <f>SUM(E2:E3)</f>
+        <v>81700</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>18302</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="1"/>
+        <v>0.22401468788249693</v>
+      </c>
+      <c r="J4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:N4" si="4">SUM(K2:K3)</f>
+        <v>38766</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="4"/>
+        <v>25626</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="4"/>
+        <v>3356</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="4"/>
+        <v>2609</v>
+      </c>
+      <c r="O4">
+        <f>SUM(O2:O3)</f>
+        <v>785811</v>
+      </c>
+      <c r="P4">
+        <f>K4+L4+M4+N4</f>
+        <v>70357</v>
+      </c>
+      <c r="Q4" s="1">
+        <f t="shared" si="2"/>
+        <v>8.9534251874814688E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>37106</v>
+      </c>
+      <c r="C7">
+        <v>7019</v>
+      </c>
+      <c r="D7">
+        <v>1162</v>
+      </c>
+      <c r="E7">
+        <v>53069</v>
+      </c>
+      <c r="F7">
+        <f>B7-C7+D7</f>
+        <v>31249</v>
+      </c>
+      <c r="G7">
+        <f>F7/E7</f>
+        <v>0.58883717424485105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>23495</v>
+      </c>
+      <c r="C8">
+        <v>17605</v>
+      </c>
+      <c r="D8">
+        <v>438</v>
+      </c>
+      <c r="E8">
+        <v>27752</v>
+      </c>
+      <c r="F8">
+        <f t="shared" ref="F8:F9" si="5">B8-C8+D8</f>
+        <v>6328</v>
+      </c>
+      <c r="G8">
+        <f t="shared" ref="G8:G9" si="6">F8/E8</f>
+        <v>0.22801960219083309</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <f t="shared" ref="B9:D9" si="7">SUM(B7:B8)</f>
+        <v>60601</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="7"/>
+        <v>24624</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="7"/>
+        <v>1600</v>
+      </c>
+      <c r="E9">
+        <f>SUM(E7:E8)</f>
+        <v>80821</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="5"/>
+        <v>37577</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="6"/>
+        <v>0.46494104255082219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12">
+        <v>19053</v>
+      </c>
+      <c r="C12">
+        <v>921</v>
+      </c>
+      <c r="D12">
+        <v>297</v>
+      </c>
+      <c r="E12">
+        <v>22207</v>
+      </c>
+      <c r="F12">
+        <f>B12-C12+D12</f>
+        <v>18429</v>
+      </c>
+      <c r="G12">
+        <f>F12/E12</f>
+        <v>0.82987346332237588</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -739,20 +2400,20 @@
         <v>0.50812243502051979</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
       <c r="B14">
-        <f t="shared" ref="B14" si="10">SUM(B12:B13)</f>
+        <f t="shared" ref="B14:D14" si="10">SUM(B12:B13)</f>
         <v>26615</v>
       </c>
       <c r="C14">
-        <f t="shared" ref="C14" si="11">SUM(C12:C13)</f>
+        <f t="shared" si="10"/>
         <v>2994</v>
       </c>
       <c r="D14">
-        <f t="shared" ref="D14" si="12">SUM(D12:D13)</f>
+        <f t="shared" si="10"/>
         <v>751</v>
       </c>
       <c r="E14">
@@ -768,7 +2429,7 @@
         <v>0.71887443589062916</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -791,7 +2452,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -816,7 +2477,7 @@
         <v>0.42664418212478922</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -833,28 +2494,28 @@
         <v>5324</v>
       </c>
       <c r="F18">
-        <f t="shared" ref="F18:F19" si="13">B18-C18+D18</f>
+        <f t="shared" ref="F18:F19" si="11">B18-C18+D18</f>
         <v>1545</v>
       </c>
       <c r="G18">
-        <f t="shared" ref="G18:G19" si="14">F18/E18</f>
+        <f t="shared" ref="G18:G19" si="12">F18/E18</f>
         <v>0.29019534184823442</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
       <c r="B19">
-        <f t="shared" ref="B19" si="15">SUM(B17:B18)</f>
+        <f t="shared" ref="B19:D19" si="13">SUM(B17:B18)</f>
         <v>5176</v>
       </c>
       <c r="C19">
-        <f t="shared" ref="C19" si="16">SUM(C17:C18)</f>
+        <f t="shared" si="13"/>
         <v>2579</v>
       </c>
       <c r="D19">
-        <f t="shared" ref="D19" si="17">SUM(D17:D18)</f>
+        <f t="shared" si="13"/>
         <v>213</v>
       </c>
       <c r="E19">
@@ -862,17 +2523,12 @@
         <v>8289</v>
       </c>
       <c r="F19">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>2810</v>
       </c>
       <c r="G19" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0.33900349861261914</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>